<commit_message>
Updated CHE model - 2025-09-14 21:54
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
+++ b/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1D71DEE-7574-4636-B281-BDC9283A1159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD324DCE-24F0-431E-B555-CC984A651C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{FFE3BE8E-FDFA-41B7-9FF5-4FA75696C0C4}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{CABA0B48-C8C3-498C-935E-806E660962CD}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="2" r:id="rId1"/>
@@ -1187,7 +1187,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01988B03-4EEA-470B-9C51-5E2B4DB646D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEA174A0-4013-4816-9504-37DC679E440A}">
   <dimension ref="B9:T21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -1877,7 +1877,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93BF5C92-F0B9-4289-BEAF-70006DED2356}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2166C5B0-3A32-45E5-9A4B-BF6AA601C99F}">
   <dimension ref="B9:T122"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHE model - 2025-09-14 21:57
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
+++ b/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD324DCE-24F0-431E-B555-CC984A651C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB5C09B4-2317-47BD-8ABD-E3E62B88976D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{CABA0B48-C8C3-498C-935E-806E660962CD}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{9FA05750-83AA-4888-9234-D20B6349F7F8}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="2" r:id="rId1"/>
@@ -1187,7 +1187,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEA174A0-4013-4816-9504-37DC679E440A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B7B7F81-D143-455D-91CA-771B6AD6EB82}">
   <dimension ref="B9:T21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -1877,7 +1877,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2166C5B0-3A32-45E5-9A4B-BF6AA601C99F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F1EB708-C8B1-490D-9502-2E92264474B0}">
   <dimension ref="B9:T122"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHE model - 2025-09-14 22:04
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
+++ b/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB5C09B4-2317-47BD-8ABD-E3E62B88976D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2B01622-6136-4133-A1EC-14E4CA3D516E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{9FA05750-83AA-4888-9234-D20B6349F7F8}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{5802AD69-08D3-4CEA-8BD8-3D300FCFC6E4}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="2" r:id="rId1"/>
@@ -1187,7 +1187,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B7B7F81-D143-455D-91CA-771B6AD6EB82}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CE0D471-7CD8-4818-8884-0175C784C52F}">
   <dimension ref="B9:T21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -1877,7 +1877,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F1EB708-C8B1-490D-9502-2E92264474B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72BDEC52-C9E7-4CC4-80C8-60BC25525279}">
   <dimension ref="B9:T122"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHE model - 2025-09-14 22:12
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
+++ b/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2B01622-6136-4133-A1EC-14E4CA3D516E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{389629CF-288F-4307-857E-E97834A13FE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{5802AD69-08D3-4CEA-8BD8-3D300FCFC6E4}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{B9143CA4-AE19-4DB6-A74C-E1DEBC660438}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="2" r:id="rId1"/>
@@ -1187,7 +1187,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CE0D471-7CD8-4818-8884-0175C784C52F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{655ED82D-9435-47E4-A638-A04E0EBEA99C}">
   <dimension ref="B9:T21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -1877,7 +1877,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72BDEC52-C9E7-4CC4-80C8-60BC25525279}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D45E02F2-CA9F-4718-B6C6-DB1FF2468136}">
   <dimension ref="B9:T122"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHE model - 2025-09-14 22:30
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
+++ b/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{389629CF-288F-4307-857E-E97834A13FE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{47F5BBA8-15C5-4A0C-8F05-9624E9883B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{B9143CA4-AE19-4DB6-A74C-E1DEBC660438}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{6986EE57-BEC8-4275-B5B1-2FED987496F6}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="2" r:id="rId1"/>
@@ -1187,7 +1187,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{655ED82D-9435-47E4-A638-A04E0EBEA99C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B0D67A9-0B37-4365-8B0C-3306D44588E8}">
   <dimension ref="B9:T21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -1877,7 +1877,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D45E02F2-CA9F-4718-B6C6-DB1FF2468136}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0851F661-CB53-4240-B318-AB0606604966}">
   <dimension ref="B9:T122"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHE model - 2025-09-14 22:38
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
+++ b/VerveStacks_CHE/vt_vervestacks_CHE_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{47F5BBA8-15C5-4A0C-8F05-9624E9883B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7CC0AE8-54A5-4132-9829-7DC94CC63F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{6986EE57-BEC8-4275-B5B1-2FED987496F6}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{2F165143-730D-49C0-8AF4-F3E2515FCC8C}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="2" r:id="rId1"/>
@@ -1187,7 +1187,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B0D67A9-0B37-4365-8B0C-3306D44588E8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AFD8EAA-C84C-4CDE-AD0E-05A6D1C7E1CA}">
   <dimension ref="B9:T21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -1877,7 +1877,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0851F661-CB53-4240-B318-AB0606604966}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A971553-86F4-41AD-A39E-10D3B48B4E62}">
   <dimension ref="B9:T122"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>